<commit_message>
Disable sheet protection so paint formulas can be edited and saved without a password.
</commit_message>
<xml_diff>
--- a/receptury-lakiery/RECEPTURY_LAKIERY.xlsx
+++ b/receptury-lakiery/RECEPTURY_LAKIERY.xlsx
@@ -1896,7 +1896,7 @@
     <row r="29">
       <c r="A29" s="22" t="inlineStr">
         <is>
-          <t>Mieszanie systemów: receptura bazowa AUTOCOLOR może zawierać pigmenty DUXONE i odwrotnie. Nie usuwaj wierszy tabel — zeruj ilość (status USUNIĘTO). Komórki złote = wpis, szare = formuła (ochrona hasłem: lakier). Źródła nazw: PDF Nexa Autocolor 2K Tint Chart oraz Duxone Tint Descriptions PL; kody z szablonów ODS.</t>
+          <t>Mieszanie systemów: receptura bazowa AUTOCOLOR może zawierać pigmenty DUXONE i odwrotnie. Nie usuwaj wierszy tabel — zeruj ilość (status USUNIĘTO). Komórki złote = wpis, szare = formuła (arkusze bez ochrony — edycja i zapis bez hasła). Źródła nazw: PDF Nexa Autocolor 2K Tint Chart oraz Duxone Tint Descriptions PL; kody z szablonów ODS.</t>
         </is>
       </c>
     </row>
@@ -1904,7 +1904,6 @@
     <row r="31"/>
     <row r="32"/>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DAF9"/>
   <mergeCells count="46">
     <mergeCell ref="I14:L14"/>
     <mergeCell ref="A29:L32"/>
@@ -12933,7 +12932,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DAF9"/>
   <autoFilter ref="A8:N194"/>
   <mergeCells count="3">
     <mergeCell ref="B4:N4"/>
@@ -13055,17 +13053,17 @@
     <row r="11">
       <c r="A11" s="34" t="inlineStr">
         <is>
-          <t>Hasło ochrony arkuszy</t>
+          <t>Ochrona arkuszy</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>lakier</t>
+          <t>WYŁĄCZONA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Hasło odblokowania formuł. Nie udostępniaj osobom edytującym tylko ilości.</t>
+          <t>Arkusze bez hasła — pełna edycja i zapis. Złote = wpis, szare = formuła.</t>
         </is>
       </c>
     </row>
@@ -13150,7 +13148,6 @@
     <row r="21"/>
     <row r="22"/>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DAF9"/>
   <mergeCells count="3">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -18778,7 +18775,6 @@
       <c r="I508" s="8" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DAF9"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
@@ -20148,7 +20144,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DAF9"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -20258,7 +20253,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DAF9"/>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
@@ -21721,7 +21715,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DAF9"/>
   <autoFilter ref="A11:J51"/>
   <mergeCells count="6">
     <mergeCell ref="A1:J1"/>
@@ -24230,7 +24223,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DAF9"/>
   <autoFilter ref="A11:P51"/>
   <mergeCells count="5">
     <mergeCell ref="A1:P1"/>
@@ -24544,7 +24536,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DAF9"/>
   <mergeCells count="3">
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A1:L1"/>
@@ -27657,7 +27648,6 @@
       <c r="C104" s="13" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DAF9"/>
   <mergeCells count="15">
     <mergeCell ref="B97:C97"/>
     <mergeCell ref="A4:H4"/>
@@ -30662,7 +30652,6 @@
       <c r="L208" s="8" t="inlineStr"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DAF9"/>
   <autoFilter ref="A8:L208"/>
   <mergeCells count="2">
     <mergeCell ref="A2:L2"/>
@@ -31118,7 +31107,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DAF9"/>
   <mergeCells count="22">
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="B7:F7"/>
@@ -41076,7 +41064,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DAF9"/>
   <autoFilter ref="A8:S115"/>
   <mergeCells count="2">
     <mergeCell ref="A2:S2"/>
@@ -47537,7 +47524,6 @@
       <c r="S87" s="51" t="inlineStr"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DAF9"/>
   <autoFilter ref="A8:S87"/>
   <mergeCells count="2">
     <mergeCell ref="A2:S2"/>

</xml_diff>

<commit_message>
Show a pigment dropdown on NR PIGMENTU based on that row's SYSTEM.
LibreOffice does not resolve INDIRECT named ranges in Validity, so lists live on LISTY and a macro opens the matching AUTOCOLOR/DUXONE list on cell click.
</commit_message>
<xml_diff>
--- a/receptury-lakiery/RECEPTURY_LAKIERY.xlsx
+++ b/receptury-lakiery/RECEPTURY_LAKIERY.xlsx
@@ -27,8 +27,12 @@
     <definedName name="Ust_Jednostka">USTAWIENIA!$B$9</definedName>
     <definedName name="Ust_Tolerancja">USTAWIENIA!$B$10</definedName>
     <definedName name="Lista_Systemow">LISTY!$A$9:$A$10</definedName>
-    <definedName name="Lista_AUTOCOLOR">BAZA_AUTOCOLOR!$C$9:$C$115</definedName>
-    <definedName name="Lista_DUXONE">BAZA_DUXONE!$C$9:$C$87</definedName>
+    <definedName name="Lista_AUTOCOLOR">LISTY!$F$9:$F$115</definedName>
+    <definedName name="Lista_DUXONE">LISTY!$H$9:$H$87</definedName>
+    <definedName name="ListaAC">LISTY!$F$9:$F$115</definedName>
+    <definedName name="ListaDX">LISTY!$H$9:$H$87</definedName>
+    <definedName name="ListaAC_NR">LISTY!$E$9:$E$115</definedName>
+    <definedName name="ListaDX_NR">LISTY!$G$9:$G$87</definedName>
     <definedName name="PigmentyKlucz">PIGMENTY!$A$9:$I$194</definedName>
     <definedName name="Meta_Nazwa">START!$C$5</definedName>
     <definedName name="Meta_Numer">START!$C$6</definedName>
@@ -1770,7 +1774,7 @@
       </c>
       <c r="C19" s="20" t="inlineStr">
         <is>
-          <t>Arkusz RECEPTURA_ORYGINALNA: wybierz SYSTEM, potem NR z listy. Ilość w gramach. Nazwa uzupełni się sama.</t>
+          <t>Arkusz RECEPTURA_ORYGINALNA: SYSTEM z listy, potem kliknij NR PIGMENTU — lista z wybranej bazy. Ilość w gramach. Nazwa uzupełni się sama.</t>
         </is>
       </c>
     </row>
@@ -20158,11 +20162,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S11"/>
+  <dimension ref="A1:S115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -20193,7 +20204,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Arkusz techniczny — listy rozwijane.</t>
+          <t>Źródło list rozwijanych NR PIGMENTU. Etykieta = kod | nazwa. Makro i Validity biorą zakres z J9/K9.</t>
         </is>
       </c>
       <c r="B2" s="4" t="n"/>
@@ -20226,6 +20237,41 @@
           <t>PRESETY_MASY_G</t>
         </is>
       </c>
+      <c r="E8" s="53" t="inlineStr">
+        <is>
+          <t>AUTOCOLOR_NR</t>
+        </is>
+      </c>
+      <c r="F8" s="53" t="inlineStr">
+        <is>
+          <t>AUTOCOLOR_LISTA</t>
+        </is>
+      </c>
+      <c r="G8" s="53" t="inlineStr">
+        <is>
+          <t>DUXONE_NR</t>
+        </is>
+      </c>
+      <c r="H8" s="53" t="inlineStr">
+        <is>
+          <t>DUXONE_LISTA</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>LICZBA</t>
+        </is>
+      </c>
+      <c r="J8" s="53" t="inlineStr">
+        <is>
+          <t>ADRES_LISTA_AC</t>
+        </is>
+      </c>
+      <c r="K8" s="53" t="inlineStr">
+        <is>
+          <t>ADRES_LISTA_DX</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -20236,6 +20282,41 @@
       <c r="C9" t="n">
         <v>100</v>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>P192-475</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>P192-475 | REGULATOR BAZY</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>DX5110</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>DX5110 | DEEP BLACK</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>wiersze listy →</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>LISTY!$F$9:$F$115</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>LISTY!$H$9:$H$87</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -20245,17 +20326,2076 @@
       </c>
       <c r="C10" t="n">
         <v>500</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>P192-528</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>P192-528 | REGULATOR UŁOŻENIA ZIARNA</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>DX5111</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>DX5111 | BLACK</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>liczba kodów →</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>107</v>
+      </c>
+      <c r="K10" t="n">
+        <v>79</v>
       </c>
     </row>
     <row r="11">
       <c r="C11" t="n">
         <v>1000</v>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>P192-5600</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>P192-5600 | REGULATOR FLOPU</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>DX5121</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>DX5121 | EFFECT BROWN</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>P420-902RT</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>P420-902RT | RT Pale White</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>DX5122</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>DX5122 | EFFECT BROWN RED</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>P420-903RT</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>P420-903RT | RT Medium Pale Yellow</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>DX5123</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>DX5123 | TRANSPARENT MAROON</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>P420-904RT</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>P420-904RT | RT Transparent Black</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>DX5126</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>DX5126 | EFFECT OCRE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>P420-905</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>P420-905 | Yellow Oxide</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>DX5130</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>DX5130 | WHITE HS</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>P420-907</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>P420-907 | Red Oxide</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>DX5134</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>DX5134 | EFFECT WHITE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>P420-908RT</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>P420-908RT | RT Russet</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>DX5136</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>DX5136 | Metallic Adjuster</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>P420-910RT</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>P420-910RT | RT Deep Blue</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>DX5161</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>DX5161 | ORANGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>P420-920</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>P420-920 | Violet</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>DX5143</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>DX5143 | RED</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>P420-926</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>P420-926 | Super Red</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>DX5144</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>DX5144 | DARK RED</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>P420-930</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>P420-930 | Lake Blue</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>DX5145</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>DX5145 | PINK RED</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>P420-933</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>P420-933 | Blue Black</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>DX5142</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>DX5142 | FLAMING RED</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>P420-938</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>P420-938 | Tone Controller</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>DX5146</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>DX5146 | MAGENTA RED</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>P420-942</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>P420-942 | Transoxide Red</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>DX5147</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>DX5147 | LIGHT RED</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>P420-952</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>P420-952 | Fast Blue</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>DX5149</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>DX5149 | BRIGHT RED</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>P420-960RT</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>P420-960RT | RT Burgundy</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>DX5155</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>DX5155</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>P420-975</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>P420-975 | Bronze Green</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>DX5162</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>DX5162 | YELLOW ORANGE (LEAD FREE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>P420-978</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>P420-978 | Brown</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>DX5163</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>DX5163 | EFFECT YELLOW (LEAD FREE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>P420-983</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>P420-983 | Strong Yellow</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>DX5166</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>DX5166 | EFFECT LIGHT YELLOW (LEAD FREE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>P425-900</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>P425-900 | HS Super White</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>DX5167</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>DX5167 | YELLOW (LEAD FREE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>P425-919</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>P425-919 | HS Clean Red Violet</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>DX5168</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>DX5168 | YELLOW BROWN</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>P425-921</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>P425-921 | HS Claret</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>DX5171</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>DX5171 | YELLOW GREEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>P425-922</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>P425-922 | HS Lagoon Blue</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>DX5172</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>DX5172 | GREEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>P425-941</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>P425-941 | HS Strong Red</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>DX5173</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>DX5173 | BRIGHT GREEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>P425-948</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>P425-948 | HS Black</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>DX5174</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>DX5174 | GOLD GREEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>P425-950</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>P425-950 | HS Jet Black</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>DX5181</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>DX5181 | GREEN BLUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>P425-954</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>P425-954 | HS Blue Green</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>DX5182</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>DX5182 | EFFECT BLUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>P425-956</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>P425-956 | HS Super Blue</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>DX5184</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>DX5184 | „Pod kątem”</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>P425-957</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>P425-957 | HS Fast Blue</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>DX5185</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>DX5185 | RED BLUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>P425-971</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>P425-971 | HS Brilliant Red</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>DX5187</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>DX5187 | VIOLET</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>P425-984</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>P425-984 | HS Medium Fine Aluminium</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>DX5188</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>DX5188 | RED VIOLET</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>P425-985</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>P425-985 | HS Fine Aluminium</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>DX5189</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>DX5189 | DARK MAGENTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>P425-986</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>P425-986 | HS Medium Aluminium</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>DX5211</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>DX5211 | Komponenty aluminiowe pod względem grubości ziarna</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>P425-987</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>P425-987 | Medium Coarse Aluminium</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>DX5212</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>DX5212 | COARSE SILVER</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>P425-988</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>P425-988 | HS Coarse Aluminium</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>DX5213</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>DX5213 | MEDIUM COARSE SILVER</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>P425-989</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>P425-989 | HS Very Coarse Aluminium</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>DX5214</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>DX5214 | MEDIUM SILVER</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>P425-991</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>P425-991 | Fine Satin Aluminium</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>DX5215</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>DX5215 | FINE SILVER</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>P425-992</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>P425-992 | HS Shining Coarse Aluminium</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>DX5216</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>DX5216</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>P425-998</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>P425-998 | HS Coarse Silver Dollar Aluminium</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>DX5217</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>DX5217 | EXTRA FINE SILVER</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>P425-EB02</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>P425-EB02 | KONWERTER BAZY DO KOMÓR SILNIKA</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>DX5221</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>DX5221 | COARSE BRIGHT SILVER</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>P426-HE02</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>P426-HE02 | Blue Frost</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>DX5223</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>DX5223 | MEDIUM BRIGHT SILVER</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>P426-HE03</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>P426-HE03 | Graphite Flake</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>DX5224</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>DX5224 | GOLD ALU</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>P426-HE04</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>P426-HE04 | Gold Flash</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>DX5225</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>DX5225 | ORANGE ALU</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>P426-HE05</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>P426-HE05 | Orange Flash</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>DX5226</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>DX5226 | FINE EXTRA BRIGHT ALU</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>P426-HE08</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>P426-HE08 | BLUE ALUMINIUM</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>DX5227</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>DX5227 | MEDIUM FINE BRIGHT ALU</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>P426-PP05</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>P426-PP05 | White Pearl</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>DX5231</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>DX5231 | SILVER PEARL</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>P426-PP06</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>P426-PP06 | Fine White Pearl</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>DX5232</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>DX5232 | FINE SILVER PEARL</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>P426-PP07</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>P426-PP07 | Blue Pearl</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>DX5241</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>DX5241 | RED PEARL</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>P426-PP08</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>P426-PP08 | Red Pearl</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>DX5242</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>DX5242 | FINE RED PEARL</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>P426-PP09</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>P426-PP09 | Gold Pearl</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>DX5243</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>DX5243 | SUPER RED PEARL</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>P426-PP10</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>P426-PP10 | Copper Pearl</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>DX5244</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>DX5244 | RED BROWN PEARL</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>P426-PP60</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>P426-PP60 | White Satin Pearl</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>DX5251</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>DX5251 | BLUE PEARL</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>P426-PP61</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>P426-PP61 | Fine Red Pearl</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>DX5261</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>DX5261 | GREEN PEARL</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>P426-PP62</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>P426-PP62 | Fine Russet Pearl</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>DX5271</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>DX5271 | GOLD PEARL</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>P426-PP63</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>P426-PP63 | Fine Blue Pearl</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>DX5281</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>DX5281 | LILAC PEARL</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>P426-PP64</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>P426-PP64 | Medium Violet Pearl</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>DX5299</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>DX5299 | UNISILVER</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>P426-PP65</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>P426-PP65 | Medium Green Pearl</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>DX5300</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>DX5300 | WHITE CRYSTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>P426-PP68</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>P426-PP68 | Orange Pearl</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>DX5301</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>DX5301 | RED CRYSTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>P429-914</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>P429-914 | HS CLEAN BLUE VIOLET</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>DX5302</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>DX5302 | BLUE CRYSTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>P429-917</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>P429-917 | HS GREEN GOLD</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>DX5303</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>DX5303 | GREEN CRYSTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>P429-923</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>P429-923 | HS Bright Maroon</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>DX5304</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>DX5304 | GOLD CRYSTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>P429-932</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>P429-932 | HS CLEAN ORGANIC ORANGE</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>DX5305</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>DX5305 | COPPER CRYSTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>P429-937</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>P429-937 | HS Pale Yellow</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>DX0112</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>DX0112 | BLACK (KOMPONENT O MAŁEJ SILE KRYCIA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>P429-961</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>P429-961 | HS Clean Magenta</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>DX0124</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>DX0124 | BROWN RED (PIGMENT O MAŁEJ SILE KRYCIA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>P429-967</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>P429-967 | HS Deep Angle Black</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>DX0132</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>DX0132 | WHITE (KOMPONENT O MAŁEJ SILE KRYCIA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>P429-972</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>P429-972 | HS Bright Amber</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>DX11</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>DX11</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>P429-973</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>P429-973 | HS Bright Orange</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>AXT100</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>AXT100</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>P429-976</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>P429-976 | HS Red Violet</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>AXT101</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>AXT101</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>P429-980</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>P429-980 | HS Speed Red</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>AXT102</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>AXT102</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>P429-981</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>P429-981 | Transparent Gold</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>AXT103</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>AXT103</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>P433-XR10</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>P433-XR10 | Crystal Silver</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>AXT104</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>AXT104</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>P433-XR11</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>P433-XR11 | Sunbeam Gold</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>AXT105</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>AXT105</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>P433-XR12</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>P433-XR12 | Radiant Red</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>AXT106</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>AXT106</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>P433-XR13</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>P433-XR13 | Galaxy Blue</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>AXT107</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>AXT107</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>P433-XR14</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>P433-XR14 | Stellar Green</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>AXT108</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>AXT108</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>P433-XR15</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>P433-XR15 | Solaris Red</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>AXT109</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>AXT109</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>P433-XR16</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>P433-XR16 | Fireside Copper</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>AXT110</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>AXT110</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>P433-XR17</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>P433-XR17 | Cosmic Turquoise</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>P433-XR18</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>P433-XR18 | Amethyst Dream</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>P434-CS32</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>P434-CS32 | Viola Fantasy</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>P434-CS33</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>P434-CS33 | Arctic Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>P434-CS34</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>P434-CS34 | Tropic Sunrise</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>P434-CS35</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>P434-CS35 | Lapis Sunlight</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>P435-GF37</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>P435-GF37 | Silver Glass</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>P440-FX20</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>P440-FX20 | CHROMAFLAIR CYAN TO PURPLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>P440-FX21</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>P440-FX21 | CHROMAFLAIR SILVER TO GREEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>P440-FX22</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>P440-FX22 | CHROMAFLAIR GREEN TO PURPLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>P440-FX23</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>P440-FX23 | CHROMAFLAIR BLUE TO RED</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>P440-FX24</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>P440-FX24 | CHROMAFLAIR MAGENTA TO GOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>P440-FX25</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>P440-FX25 | CHROMAFLAIR GOLD TO SILVER</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>P440-FX26</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>P440-FX26 | CHROMAFLAIR RED TO GOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>P440-FX51</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>P440-FX51 | Silver Flair</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>P440-LM01</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>P440-LM01 | LIQUID METAL SUPER FINE</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>P450-EC50</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>P450-EC50 | BRILLIANT RED</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>P420-982</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>P420-982 | Trans Oxide Yellow</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>VM4370</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>VM4370 | Super Fine Liquid Metal</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>P426-HE07</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>P426-HE07 | Blue Flash</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>P434-CS31</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>P434-CS31 | Autumn Mystery</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>VM4987</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>VM4987 | Cyan to Purple</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>VM4988</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>VM4988 | Silver to Green</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>VM4989</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>VM4989 | Green to Purple</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>VM4990</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>VM4990 | Blue to Red</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>VM4991</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>VM4991 | Magenta to Gold</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>VM4994</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>VM4994 | Gold to Silver</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>VM4995</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>VM4995 | Red to Gold</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -20272,7 +22412,7 @@
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -20427,7 +22567,7 @@
     <row r="7">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>Wpisz SYSTEM (AUTOCOLOR lub DUXONE), potem NR z listy zależnej. Możesz mieszać systemy. Ilość ≥ 0. Ten sam klucz dwa razy = DUPLIKAT (zsumuj ilości).</t>
+          <t>Najpierw SYSTEM (AUTOCOLOR / DUXONE) z listy, potem kliknij NR PIGMENTU — otworzy się lista z tej bazy. Każdy wiersz ma własny SYSTEM (można mieszać). Po wyborze numeru nazwa i jednostka uzupełnią się same. Ilość ≥ 0. Ten sam klucz dwa razy = DUPLIKAT (zsumuj ilości).</t>
         </is>
       </c>
     </row>
@@ -20516,7 +22656,7 @@
       </c>
       <c r="H12" s="8" t="n"/>
       <c r="I12" s="14">
-        <f>IF(C12="","",B12&amp;"|"&amp;C12)</f>
+        <f>IF(C12="","",B12&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C12)),TRIM(LEFT(C12,FIND(" | ",C12)-1)),C12))</f>
         <v/>
       </c>
       <c r="J12" s="14">
@@ -20556,7 +22696,7 @@
       </c>
       <c r="H13" s="8" t="n"/>
       <c r="I13" s="14">
-        <f>IF(C13="","",B13&amp;"|"&amp;C13)</f>
+        <f>IF(C13="","",B13&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C13)),TRIM(LEFT(C13,FIND(" | ",C13)-1)),C13))</f>
         <v/>
       </c>
       <c r="J13" s="14">
@@ -20596,7 +22736,7 @@
       </c>
       <c r="H14" s="8" t="n"/>
       <c r="I14" s="14">
-        <f>IF(C14="","",B14&amp;"|"&amp;C14)</f>
+        <f>IF(C14="","",B14&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C14)),TRIM(LEFT(C14,FIND(" | ",C14)-1)),C14))</f>
         <v/>
       </c>
       <c r="J14" s="14">
@@ -20626,7 +22766,7 @@
       </c>
       <c r="H15" s="8" t="n"/>
       <c r="I15" s="14">
-        <f>IF(C15="","",B15&amp;"|"&amp;C15)</f>
+        <f>IF(C15="","",B15&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C15)),TRIM(LEFT(C15,FIND(" | ",C15)-1)),C15))</f>
         <v/>
       </c>
       <c r="J15" s="14">
@@ -20656,7 +22796,7 @@
       </c>
       <c r="H16" s="8" t="n"/>
       <c r="I16" s="14">
-        <f>IF(C16="","",B16&amp;"|"&amp;C16)</f>
+        <f>IF(C16="","",B16&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C16)),TRIM(LEFT(C16,FIND(" | ",C16)-1)),C16))</f>
         <v/>
       </c>
       <c r="J16" s="14">
@@ -20686,7 +22826,7 @@
       </c>
       <c r="H17" s="8" t="n"/>
       <c r="I17" s="14">
-        <f>IF(C17="","",B17&amp;"|"&amp;C17)</f>
+        <f>IF(C17="","",B17&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C17)),TRIM(LEFT(C17,FIND(" | ",C17)-1)),C17))</f>
         <v/>
       </c>
       <c r="J17" s="14">
@@ -20716,7 +22856,7 @@
       </c>
       <c r="H18" s="8" t="n"/>
       <c r="I18" s="14">
-        <f>IF(C18="","",B18&amp;"|"&amp;C18)</f>
+        <f>IF(C18="","",B18&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C18)),TRIM(LEFT(C18,FIND(" | ",C18)-1)),C18))</f>
         <v/>
       </c>
       <c r="J18" s="14">
@@ -20746,7 +22886,7 @@
       </c>
       <c r="H19" s="8" t="n"/>
       <c r="I19" s="14">
-        <f>IF(C19="","",B19&amp;"|"&amp;C19)</f>
+        <f>IF(C19="","",B19&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C19)),TRIM(LEFT(C19,FIND(" | ",C19)-1)),C19))</f>
         <v/>
       </c>
       <c r="J19" s="14">
@@ -20776,7 +22916,7 @@
       </c>
       <c r="H20" s="8" t="n"/>
       <c r="I20" s="14">
-        <f>IF(C20="","",B20&amp;"|"&amp;C20)</f>
+        <f>IF(C20="","",B20&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C20)),TRIM(LEFT(C20,FIND(" | ",C20)-1)),C20))</f>
         <v/>
       </c>
       <c r="J20" s="14">
@@ -20806,7 +22946,7 @@
       </c>
       <c r="H21" s="8" t="n"/>
       <c r="I21" s="14">
-        <f>IF(C21="","",B21&amp;"|"&amp;C21)</f>
+        <f>IF(C21="","",B21&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C21)),TRIM(LEFT(C21,FIND(" | ",C21)-1)),C21))</f>
         <v/>
       </c>
       <c r="J21" s="14">
@@ -20836,7 +22976,7 @@
       </c>
       <c r="H22" s="8" t="n"/>
       <c r="I22" s="14">
-        <f>IF(C22="","",B22&amp;"|"&amp;C22)</f>
+        <f>IF(C22="","",B22&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C22)),TRIM(LEFT(C22,FIND(" | ",C22)-1)),C22))</f>
         <v/>
       </c>
       <c r="J22" s="14">
@@ -20866,7 +23006,7 @@
       </c>
       <c r="H23" s="8" t="n"/>
       <c r="I23" s="14">
-        <f>IF(C23="","",B23&amp;"|"&amp;C23)</f>
+        <f>IF(C23="","",B23&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C23)),TRIM(LEFT(C23,FIND(" | ",C23)-1)),C23))</f>
         <v/>
       </c>
       <c r="J23" s="14">
@@ -20896,7 +23036,7 @@
       </c>
       <c r="H24" s="8" t="n"/>
       <c r="I24" s="14">
-        <f>IF(C24="","",B24&amp;"|"&amp;C24)</f>
+        <f>IF(C24="","",B24&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C24)),TRIM(LEFT(C24,FIND(" | ",C24)-1)),C24))</f>
         <v/>
       </c>
       <c r="J24" s="14">
@@ -20926,7 +23066,7 @@
       </c>
       <c r="H25" s="8" t="n"/>
       <c r="I25" s="14">
-        <f>IF(C25="","",B25&amp;"|"&amp;C25)</f>
+        <f>IF(C25="","",B25&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C25)),TRIM(LEFT(C25,FIND(" | ",C25)-1)),C25))</f>
         <v/>
       </c>
       <c r="J25" s="14">
@@ -20956,7 +23096,7 @@
       </c>
       <c r="H26" s="8" t="n"/>
       <c r="I26" s="14">
-        <f>IF(C26="","",B26&amp;"|"&amp;C26)</f>
+        <f>IF(C26="","",B26&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C26)),TRIM(LEFT(C26,FIND(" | ",C26)-1)),C26))</f>
         <v/>
       </c>
       <c r="J26" s="14">
@@ -20986,7 +23126,7 @@
       </c>
       <c r="H27" s="8" t="n"/>
       <c r="I27" s="14">
-        <f>IF(C27="","",B27&amp;"|"&amp;C27)</f>
+        <f>IF(C27="","",B27&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C27)),TRIM(LEFT(C27,FIND(" | ",C27)-1)),C27))</f>
         <v/>
       </c>
       <c r="J27" s="14">
@@ -21016,7 +23156,7 @@
       </c>
       <c r="H28" s="8" t="n"/>
       <c r="I28" s="14">
-        <f>IF(C28="","",B28&amp;"|"&amp;C28)</f>
+        <f>IF(C28="","",B28&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C28)),TRIM(LEFT(C28,FIND(" | ",C28)-1)),C28))</f>
         <v/>
       </c>
       <c r="J28" s="14">
@@ -21046,7 +23186,7 @@
       </c>
       <c r="H29" s="8" t="n"/>
       <c r="I29" s="14">
-        <f>IF(C29="","",B29&amp;"|"&amp;C29)</f>
+        <f>IF(C29="","",B29&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C29)),TRIM(LEFT(C29,FIND(" | ",C29)-1)),C29))</f>
         <v/>
       </c>
       <c r="J29" s="14">
@@ -21076,7 +23216,7 @@
       </c>
       <c r="H30" s="8" t="n"/>
       <c r="I30" s="14">
-        <f>IF(C30="","",B30&amp;"|"&amp;C30)</f>
+        <f>IF(C30="","",B30&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C30)),TRIM(LEFT(C30,FIND(" | ",C30)-1)),C30))</f>
         <v/>
       </c>
       <c r="J30" s="14">
@@ -21106,7 +23246,7 @@
       </c>
       <c r="H31" s="8" t="n"/>
       <c r="I31" s="14">
-        <f>IF(C31="","",B31&amp;"|"&amp;C31)</f>
+        <f>IF(C31="","",B31&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C31)),TRIM(LEFT(C31,FIND(" | ",C31)-1)),C31))</f>
         <v/>
       </c>
       <c r="J31" s="14">
@@ -21136,7 +23276,7 @@
       </c>
       <c r="H32" s="8" t="n"/>
       <c r="I32" s="14">
-        <f>IF(C32="","",B32&amp;"|"&amp;C32)</f>
+        <f>IF(C32="","",B32&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C32)),TRIM(LEFT(C32,FIND(" | ",C32)-1)),C32))</f>
         <v/>
       </c>
       <c r="J32" s="14">
@@ -21166,7 +23306,7 @@
       </c>
       <c r="H33" s="8" t="n"/>
       <c r="I33" s="14">
-        <f>IF(C33="","",B33&amp;"|"&amp;C33)</f>
+        <f>IF(C33="","",B33&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C33)),TRIM(LEFT(C33,FIND(" | ",C33)-1)),C33))</f>
         <v/>
       </c>
       <c r="J33" s="14">
@@ -21196,7 +23336,7 @@
       </c>
       <c r="H34" s="8" t="n"/>
       <c r="I34" s="14">
-        <f>IF(C34="","",B34&amp;"|"&amp;C34)</f>
+        <f>IF(C34="","",B34&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C34)),TRIM(LEFT(C34,FIND(" | ",C34)-1)),C34))</f>
         <v/>
       </c>
       <c r="J34" s="14">
@@ -21226,7 +23366,7 @@
       </c>
       <c r="H35" s="8" t="n"/>
       <c r="I35" s="14">
-        <f>IF(C35="","",B35&amp;"|"&amp;C35)</f>
+        <f>IF(C35="","",B35&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C35)),TRIM(LEFT(C35,FIND(" | ",C35)-1)),C35))</f>
         <v/>
       </c>
       <c r="J35" s="14">
@@ -21256,7 +23396,7 @@
       </c>
       <c r="H36" s="8" t="n"/>
       <c r="I36" s="14">
-        <f>IF(C36="","",B36&amp;"|"&amp;C36)</f>
+        <f>IF(C36="","",B36&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C36)),TRIM(LEFT(C36,FIND(" | ",C36)-1)),C36))</f>
         <v/>
       </c>
       <c r="J36" s="14">
@@ -21286,7 +23426,7 @@
       </c>
       <c r="H37" s="8" t="n"/>
       <c r="I37" s="14">
-        <f>IF(C37="","",B37&amp;"|"&amp;C37)</f>
+        <f>IF(C37="","",B37&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C37)),TRIM(LEFT(C37,FIND(" | ",C37)-1)),C37))</f>
         <v/>
       </c>
       <c r="J37" s="14">
@@ -21316,7 +23456,7 @@
       </c>
       <c r="H38" s="8" t="n"/>
       <c r="I38" s="14">
-        <f>IF(C38="","",B38&amp;"|"&amp;C38)</f>
+        <f>IF(C38="","",B38&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C38)),TRIM(LEFT(C38,FIND(" | ",C38)-1)),C38))</f>
         <v/>
       </c>
       <c r="J38" s="14">
@@ -21346,7 +23486,7 @@
       </c>
       <c r="H39" s="8" t="n"/>
       <c r="I39" s="14">
-        <f>IF(C39="","",B39&amp;"|"&amp;C39)</f>
+        <f>IF(C39="","",B39&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C39)),TRIM(LEFT(C39,FIND(" | ",C39)-1)),C39))</f>
         <v/>
       </c>
       <c r="J39" s="14">
@@ -21376,7 +23516,7 @@
       </c>
       <c r="H40" s="8" t="n"/>
       <c r="I40" s="14">
-        <f>IF(C40="","",B40&amp;"|"&amp;C40)</f>
+        <f>IF(C40="","",B40&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C40)),TRIM(LEFT(C40,FIND(" | ",C40)-1)),C40))</f>
         <v/>
       </c>
       <c r="J40" s="14">
@@ -21406,7 +23546,7 @@
       </c>
       <c r="H41" s="8" t="n"/>
       <c r="I41" s="14">
-        <f>IF(C41="","",B41&amp;"|"&amp;C41)</f>
+        <f>IF(C41="","",B41&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C41)),TRIM(LEFT(C41,FIND(" | ",C41)-1)),C41))</f>
         <v/>
       </c>
       <c r="J41" s="14">
@@ -21436,7 +23576,7 @@
       </c>
       <c r="H42" s="8" t="n"/>
       <c r="I42" s="14">
-        <f>IF(C42="","",B42&amp;"|"&amp;C42)</f>
+        <f>IF(C42="","",B42&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C42)),TRIM(LEFT(C42,FIND(" | ",C42)-1)),C42))</f>
         <v/>
       </c>
       <c r="J42" s="14">
@@ -21466,7 +23606,7 @@
       </c>
       <c r="H43" s="8" t="n"/>
       <c r="I43" s="14">
-        <f>IF(C43="","",B43&amp;"|"&amp;C43)</f>
+        <f>IF(C43="","",B43&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C43)),TRIM(LEFT(C43,FIND(" | ",C43)-1)),C43))</f>
         <v/>
       </c>
       <c r="J43" s="14">
@@ -21496,7 +23636,7 @@
       </c>
       <c r="H44" s="8" t="n"/>
       <c r="I44" s="14">
-        <f>IF(C44="","",B44&amp;"|"&amp;C44)</f>
+        <f>IF(C44="","",B44&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C44)),TRIM(LEFT(C44,FIND(" | ",C44)-1)),C44))</f>
         <v/>
       </c>
       <c r="J44" s="14">
@@ -21526,7 +23666,7 @@
       </c>
       <c r="H45" s="8" t="n"/>
       <c r="I45" s="14">
-        <f>IF(C45="","",B45&amp;"|"&amp;C45)</f>
+        <f>IF(C45="","",B45&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C45)),TRIM(LEFT(C45,FIND(" | ",C45)-1)),C45))</f>
         <v/>
       </c>
       <c r="J45" s="14">
@@ -21556,7 +23696,7 @@
       </c>
       <c r="H46" s="8" t="n"/>
       <c r="I46" s="14">
-        <f>IF(C46="","",B46&amp;"|"&amp;C46)</f>
+        <f>IF(C46="","",B46&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C46)),TRIM(LEFT(C46,FIND(" | ",C46)-1)),C46))</f>
         <v/>
       </c>
       <c r="J46" s="14">
@@ -21586,7 +23726,7 @@
       </c>
       <c r="H47" s="8" t="n"/>
       <c r="I47" s="14">
-        <f>IF(C47="","",B47&amp;"|"&amp;C47)</f>
+        <f>IF(C47="","",B47&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C47)),TRIM(LEFT(C47,FIND(" | ",C47)-1)),C47))</f>
         <v/>
       </c>
       <c r="J47" s="14">
@@ -21616,7 +23756,7 @@
       </c>
       <c r="H48" s="8" t="n"/>
       <c r="I48" s="14">
-        <f>IF(C48="","",B48&amp;"|"&amp;C48)</f>
+        <f>IF(C48="","",B48&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C48)),TRIM(LEFT(C48,FIND(" | ",C48)-1)),C48))</f>
         <v/>
       </c>
       <c r="J48" s="14">
@@ -21646,7 +23786,7 @@
       </c>
       <c r="H49" s="8" t="n"/>
       <c r="I49" s="14">
-        <f>IF(C49="","",B49&amp;"|"&amp;C49)</f>
+        <f>IF(C49="","",B49&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C49)),TRIM(LEFT(C49,FIND(" | ",C49)-1)),C49))</f>
         <v/>
       </c>
       <c r="J49" s="14">
@@ -21676,7 +23816,7 @@
       </c>
       <c r="H50" s="8" t="n"/>
       <c r="I50" s="14">
-        <f>IF(C50="","",B50&amp;"|"&amp;C50)</f>
+        <f>IF(C50="","",B50&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C50)),TRIM(LEFT(C50,FIND(" | ",C50)-1)),C50))</f>
         <v/>
       </c>
       <c r="J50" s="14">
@@ -21706,7 +23846,7 @@
       </c>
       <c r="H51" s="8" t="n"/>
       <c r="I51" s="14">
-        <f>IF(C51="","",B51&amp;"|"&amp;C51)</f>
+        <f>IF(C51="","",B51&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C51)),TRIM(LEFT(C51,FIND(" | ",C51)-1)),C51))</f>
         <v/>
       </c>
       <c r="J51" s="14">
@@ -21739,8 +23879,8 @@
     <dataValidation sqref="E12:E51" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Ilość ujemna" error="Ilość nie może być ujemna." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="C12:C51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=INDIRECT("Lista_"&amp;B12)</formula1>
+    <dataValidation sqref="C12:C51" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="NR PIGMENTU" prompt="Wybierz pigment z listy (baza = SYSTEM w tym wierszu). Nie wpisuj kodu ręcznie." type="list">
+      <formula1>=INDIRECT(IF($B12="DUXONE",LISTY!$K$9,LISTY!$J$9))</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -21758,7 +23898,7 @@
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -21945,7 +24085,7 @@
     <row r="7">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>Kolumny złote: SYSTEM, NR, ILOŚĆ WŁASNA, UWAGI. ILOŚĆ DO ZWAŻENIA = ilość własna × masa docelowa / masa własna (przeliczenie na 100 g / 500 g / 1 kg / dowolna). STATUS: BEZ ZMIAN / ZWIĘKSZONO / ZMNIEJSZONO / DODANO / USUNIĘTO. Usunięcie = ilość własna 0 przy ilości oryginalnej &gt; 0.</t>
+          <t>Kolumny złote: SYSTEM, NR, ILOŚĆ WŁASNA, UWAGI. Kliknij NR PIGMENTU — lista z bazy SYSTEM w tym wierszu (można mieszać AUTOCOLOR i DUXONE). ILOŚĆ DO ZWAŻENIA = ilość własna × masa docelowa / masa własna (przeliczenie na 100 g / 500 g / 1 kg / dowolna). STATUS: BEZ ZMIAN / ZWIĘKSZONO / ZMNIEJSZONO / DODANO / USUNIĘTO. Usunięcie = ilość własna 0 przy ilości oryginalnej &gt; 0.</t>
         </is>
       </c>
     </row>
@@ -22092,7 +24232,7 @@
         <v/>
       </c>
       <c r="P12" s="14">
-        <f>IF(C12="","",B12&amp;"|"&amp;C12)</f>
+        <f>IF(C12="","",B12&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C12)),TRIM(LEFT(C12,FIND(" | ",C12)-1)),C12))</f>
         <v/>
       </c>
     </row>
@@ -22156,7 +24296,7 @@
         <v/>
       </c>
       <c r="P13" s="14">
-        <f>IF(C13="","",B13&amp;"|"&amp;C13)</f>
+        <f>IF(C13="","",B13&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C13)),TRIM(LEFT(C13,FIND(" | ",C13)-1)),C13))</f>
         <v/>
       </c>
     </row>
@@ -22220,7 +24360,7 @@
         <v/>
       </c>
       <c r="P14" s="14">
-        <f>IF(C14="","",B14&amp;"|"&amp;C14)</f>
+        <f>IF(C14="","",B14&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C14)),TRIM(LEFT(C14,FIND(" | ",C14)-1)),C14))</f>
         <v/>
       </c>
     </row>
@@ -22274,7 +24414,7 @@
         <v/>
       </c>
       <c r="P15" s="14">
-        <f>IF(C15="","",B15&amp;"|"&amp;C15)</f>
+        <f>IF(C15="","",B15&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C15)),TRIM(LEFT(C15,FIND(" | ",C15)-1)),C15))</f>
         <v/>
       </c>
     </row>
@@ -22328,7 +24468,7 @@
         <v/>
       </c>
       <c r="P16" s="14">
-        <f>IF(C16="","",B16&amp;"|"&amp;C16)</f>
+        <f>IF(C16="","",B16&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C16)),TRIM(LEFT(C16,FIND(" | ",C16)-1)),C16))</f>
         <v/>
       </c>
     </row>
@@ -22382,7 +24522,7 @@
         <v/>
       </c>
       <c r="P17" s="14">
-        <f>IF(C17="","",B17&amp;"|"&amp;C17)</f>
+        <f>IF(C17="","",B17&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C17)),TRIM(LEFT(C17,FIND(" | ",C17)-1)),C17))</f>
         <v/>
       </c>
     </row>
@@ -22436,7 +24576,7 @@
         <v/>
       </c>
       <c r="P18" s="14">
-        <f>IF(C18="","",B18&amp;"|"&amp;C18)</f>
+        <f>IF(C18="","",B18&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C18)),TRIM(LEFT(C18,FIND(" | ",C18)-1)),C18))</f>
         <v/>
       </c>
     </row>
@@ -22490,7 +24630,7 @@
         <v/>
       </c>
       <c r="P19" s="14">
-        <f>IF(C19="","",B19&amp;"|"&amp;C19)</f>
+        <f>IF(C19="","",B19&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C19)),TRIM(LEFT(C19,FIND(" | ",C19)-1)),C19))</f>
         <v/>
       </c>
     </row>
@@ -22544,7 +24684,7 @@
         <v/>
       </c>
       <c r="P20" s="14">
-        <f>IF(C20="","",B20&amp;"|"&amp;C20)</f>
+        <f>IF(C20="","",B20&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C20)),TRIM(LEFT(C20,FIND(" | ",C20)-1)),C20))</f>
         <v/>
       </c>
     </row>
@@ -22598,7 +24738,7 @@
         <v/>
       </c>
       <c r="P21" s="14">
-        <f>IF(C21="","",B21&amp;"|"&amp;C21)</f>
+        <f>IF(C21="","",B21&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C21)),TRIM(LEFT(C21,FIND(" | ",C21)-1)),C21))</f>
         <v/>
       </c>
     </row>
@@ -22652,7 +24792,7 @@
         <v/>
       </c>
       <c r="P22" s="14">
-        <f>IF(C22="","",B22&amp;"|"&amp;C22)</f>
+        <f>IF(C22="","",B22&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C22)),TRIM(LEFT(C22,FIND(" | ",C22)-1)),C22))</f>
         <v/>
       </c>
     </row>
@@ -22706,7 +24846,7 @@
         <v/>
       </c>
       <c r="P23" s="14">
-        <f>IF(C23="","",B23&amp;"|"&amp;C23)</f>
+        <f>IF(C23="","",B23&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C23)),TRIM(LEFT(C23,FIND(" | ",C23)-1)),C23))</f>
         <v/>
       </c>
     </row>
@@ -22760,7 +24900,7 @@
         <v/>
       </c>
       <c r="P24" s="14">
-        <f>IF(C24="","",B24&amp;"|"&amp;C24)</f>
+        <f>IF(C24="","",B24&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C24)),TRIM(LEFT(C24,FIND(" | ",C24)-1)),C24))</f>
         <v/>
       </c>
     </row>
@@ -22814,7 +24954,7 @@
         <v/>
       </c>
       <c r="P25" s="14">
-        <f>IF(C25="","",B25&amp;"|"&amp;C25)</f>
+        <f>IF(C25="","",B25&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C25)),TRIM(LEFT(C25,FIND(" | ",C25)-1)),C25))</f>
         <v/>
       </c>
     </row>
@@ -22868,7 +25008,7 @@
         <v/>
       </c>
       <c r="P26" s="14">
-        <f>IF(C26="","",B26&amp;"|"&amp;C26)</f>
+        <f>IF(C26="","",B26&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C26)),TRIM(LEFT(C26,FIND(" | ",C26)-1)),C26))</f>
         <v/>
       </c>
     </row>
@@ -22922,7 +25062,7 @@
         <v/>
       </c>
       <c r="P27" s="14">
-        <f>IF(C27="","",B27&amp;"|"&amp;C27)</f>
+        <f>IF(C27="","",B27&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C27)),TRIM(LEFT(C27,FIND(" | ",C27)-1)),C27))</f>
         <v/>
       </c>
     </row>
@@ -22976,7 +25116,7 @@
         <v/>
       </c>
       <c r="P28" s="14">
-        <f>IF(C28="","",B28&amp;"|"&amp;C28)</f>
+        <f>IF(C28="","",B28&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C28)),TRIM(LEFT(C28,FIND(" | ",C28)-1)),C28))</f>
         <v/>
       </c>
     </row>
@@ -23030,7 +25170,7 @@
         <v/>
       </c>
       <c r="P29" s="14">
-        <f>IF(C29="","",B29&amp;"|"&amp;C29)</f>
+        <f>IF(C29="","",B29&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C29)),TRIM(LEFT(C29,FIND(" | ",C29)-1)),C29))</f>
         <v/>
       </c>
     </row>
@@ -23084,7 +25224,7 @@
         <v/>
       </c>
       <c r="P30" s="14">
-        <f>IF(C30="","",B30&amp;"|"&amp;C30)</f>
+        <f>IF(C30="","",B30&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C30)),TRIM(LEFT(C30,FIND(" | ",C30)-1)),C30))</f>
         <v/>
       </c>
     </row>
@@ -23138,7 +25278,7 @@
         <v/>
       </c>
       <c r="P31" s="14">
-        <f>IF(C31="","",B31&amp;"|"&amp;C31)</f>
+        <f>IF(C31="","",B31&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C31)),TRIM(LEFT(C31,FIND(" | ",C31)-1)),C31))</f>
         <v/>
       </c>
     </row>
@@ -23192,7 +25332,7 @@
         <v/>
       </c>
       <c r="P32" s="14">
-        <f>IF(C32="","",B32&amp;"|"&amp;C32)</f>
+        <f>IF(C32="","",B32&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C32)),TRIM(LEFT(C32,FIND(" | ",C32)-1)),C32))</f>
         <v/>
       </c>
     </row>
@@ -23246,7 +25386,7 @@
         <v/>
       </c>
       <c r="P33" s="14">
-        <f>IF(C33="","",B33&amp;"|"&amp;C33)</f>
+        <f>IF(C33="","",B33&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C33)),TRIM(LEFT(C33,FIND(" | ",C33)-1)),C33))</f>
         <v/>
       </c>
     </row>
@@ -23300,7 +25440,7 @@
         <v/>
       </c>
       <c r="P34" s="14">
-        <f>IF(C34="","",B34&amp;"|"&amp;C34)</f>
+        <f>IF(C34="","",B34&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C34)),TRIM(LEFT(C34,FIND(" | ",C34)-1)),C34))</f>
         <v/>
       </c>
     </row>
@@ -23354,7 +25494,7 @@
         <v/>
       </c>
       <c r="P35" s="14">
-        <f>IF(C35="","",B35&amp;"|"&amp;C35)</f>
+        <f>IF(C35="","",B35&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C35)),TRIM(LEFT(C35,FIND(" | ",C35)-1)),C35))</f>
         <v/>
       </c>
     </row>
@@ -23408,7 +25548,7 @@
         <v/>
       </c>
       <c r="P36" s="14">
-        <f>IF(C36="","",B36&amp;"|"&amp;C36)</f>
+        <f>IF(C36="","",B36&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C36)),TRIM(LEFT(C36,FIND(" | ",C36)-1)),C36))</f>
         <v/>
       </c>
     </row>
@@ -23462,7 +25602,7 @@
         <v/>
       </c>
       <c r="P37" s="14">
-        <f>IF(C37="","",B37&amp;"|"&amp;C37)</f>
+        <f>IF(C37="","",B37&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C37)),TRIM(LEFT(C37,FIND(" | ",C37)-1)),C37))</f>
         <v/>
       </c>
     </row>
@@ -23516,7 +25656,7 @@
         <v/>
       </c>
       <c r="P38" s="14">
-        <f>IF(C38="","",B38&amp;"|"&amp;C38)</f>
+        <f>IF(C38="","",B38&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C38)),TRIM(LEFT(C38,FIND(" | ",C38)-1)),C38))</f>
         <v/>
       </c>
     </row>
@@ -23570,7 +25710,7 @@
         <v/>
       </c>
       <c r="P39" s="14">
-        <f>IF(C39="","",B39&amp;"|"&amp;C39)</f>
+        <f>IF(C39="","",B39&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C39)),TRIM(LEFT(C39,FIND(" | ",C39)-1)),C39))</f>
         <v/>
       </c>
     </row>
@@ -23624,7 +25764,7 @@
         <v/>
       </c>
       <c r="P40" s="14">
-        <f>IF(C40="","",B40&amp;"|"&amp;C40)</f>
+        <f>IF(C40="","",B40&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C40)),TRIM(LEFT(C40,FIND(" | ",C40)-1)),C40))</f>
         <v/>
       </c>
     </row>
@@ -23678,7 +25818,7 @@
         <v/>
       </c>
       <c r="P41" s="14">
-        <f>IF(C41="","",B41&amp;"|"&amp;C41)</f>
+        <f>IF(C41="","",B41&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C41)),TRIM(LEFT(C41,FIND(" | ",C41)-1)),C41))</f>
         <v/>
       </c>
     </row>
@@ -23732,7 +25872,7 @@
         <v/>
       </c>
       <c r="P42" s="14">
-        <f>IF(C42="","",B42&amp;"|"&amp;C42)</f>
+        <f>IF(C42="","",B42&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C42)),TRIM(LEFT(C42,FIND(" | ",C42)-1)),C42))</f>
         <v/>
       </c>
     </row>
@@ -23786,7 +25926,7 @@
         <v/>
       </c>
       <c r="P43" s="14">
-        <f>IF(C43="","",B43&amp;"|"&amp;C43)</f>
+        <f>IF(C43="","",B43&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C43)),TRIM(LEFT(C43,FIND(" | ",C43)-1)),C43))</f>
         <v/>
       </c>
     </row>
@@ -23840,7 +25980,7 @@
         <v/>
       </c>
       <c r="P44" s="14">
-        <f>IF(C44="","",B44&amp;"|"&amp;C44)</f>
+        <f>IF(C44="","",B44&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C44)),TRIM(LEFT(C44,FIND(" | ",C44)-1)),C44))</f>
         <v/>
       </c>
     </row>
@@ -23894,7 +26034,7 @@
         <v/>
       </c>
       <c r="P45" s="14">
-        <f>IF(C45="","",B45&amp;"|"&amp;C45)</f>
+        <f>IF(C45="","",B45&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C45)),TRIM(LEFT(C45,FIND(" | ",C45)-1)),C45))</f>
         <v/>
       </c>
     </row>
@@ -23948,7 +26088,7 @@
         <v/>
       </c>
       <c r="P46" s="14">
-        <f>IF(C46="","",B46&amp;"|"&amp;C46)</f>
+        <f>IF(C46="","",B46&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C46)),TRIM(LEFT(C46,FIND(" | ",C46)-1)),C46))</f>
         <v/>
       </c>
     </row>
@@ -24002,7 +26142,7 @@
         <v/>
       </c>
       <c r="P47" s="14">
-        <f>IF(C47="","",B47&amp;"|"&amp;C47)</f>
+        <f>IF(C47="","",B47&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C47)),TRIM(LEFT(C47,FIND(" | ",C47)-1)),C47))</f>
         <v/>
       </c>
     </row>
@@ -24056,7 +26196,7 @@
         <v/>
       </c>
       <c r="P48" s="14">
-        <f>IF(C48="","",B48&amp;"|"&amp;C48)</f>
+        <f>IF(C48="","",B48&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C48)),TRIM(LEFT(C48,FIND(" | ",C48)-1)),C48))</f>
         <v/>
       </c>
     </row>
@@ -24110,7 +26250,7 @@
         <v/>
       </c>
       <c r="P49" s="14">
-        <f>IF(C49="","",B49&amp;"|"&amp;C49)</f>
+        <f>IF(C49="","",B49&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C49)),TRIM(LEFT(C49,FIND(" | ",C49)-1)),C49))</f>
         <v/>
       </c>
     </row>
@@ -24164,7 +26304,7 @@
         <v/>
       </c>
       <c r="P50" s="14">
-        <f>IF(C50="","",B50&amp;"|"&amp;C50)</f>
+        <f>IF(C50="","",B50&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C50)),TRIM(LEFT(C50,FIND(" | ",C50)-1)),C50))</f>
         <v/>
       </c>
     </row>
@@ -24218,7 +26358,7 @@
         <v/>
       </c>
       <c r="P51" s="14">
-        <f>IF(C51="","",B51&amp;"|"&amp;C51)</f>
+        <f>IF(C51="","",B51&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",C51)),TRIM(LEFT(C51,FIND(" | ",C51)-1)),C51))</f>
         <v/>
       </c>
     </row>
@@ -24265,8 +26405,8 @@
     <dataValidation sqref="F12:F51" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Ilość ujemna" error="Ilość nie może być ujemna." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="C12:C51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=INDIRECT("Lista_"&amp;B12)</formula1>
+    <dataValidation sqref="C12:C51" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="NR PIGMENTU" prompt="Wybierz pigment z listy (baza = SYSTEM w tym wierszu). Nie wpisuj kodu ręcznie." type="list">
+      <formula1>=INDIRECT(IF($B12="DUXONE",LISTY!$K$9,LISTY!$J$9))</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -30755,7 +32895,7 @@
         </is>
       </c>
       <c r="B6" s="14">
-        <f>IF(OR(B4="",B5=""),"",B4&amp;"|"&amp;B5)</f>
+        <f>IF(OR(B4="",B5=""),"",B4&amp;"|"&amp;IF(ISNUMBER(FIND(" | ",B5)),TRIM(LEFT(B5,FIND(" | ",B5)-1)),B5))</f>
         <v/>
       </c>
       <c r="C6">
@@ -31135,8 +33275,8 @@
     <dataValidation sqref="B4" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Niedozwolona wartość" error="Wybierz wartość z listy." promptTitle="Wybór" prompt="Wybierz z listy rozwijanej." type="list">
       <formula1>=Lista_Systemow</formula1>
     </dataValidation>
-    <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=INDIRECT("Lista_"&amp;B4)</formula1>
+    <dataValidation sqref="B5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="NR PIGMENTU" prompt="Wybierz pigment z listy (baza = SYSTEM w tym wierszu). Nie wpisuj kodu ręcznie." type="list">
+      <formula1>=INDIRECT(IF($B4="DUXONE",LISTY!$K$9,LISTY!$J$9))</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Open a native Windows file dialog when importing a recipe from PDF.
</commit_message>
<xml_diff>
--- a/receptury-lakiery/RECEPTURY_LAKIERY.xlsx
+++ b/receptury-lakiery/RECEPTURY_LAKIERY.xlsx
@@ -1841,7 +1841,7 @@
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>Makro ImportujZPdf: wskaż PDF receptury Autocolor/Duxone (kody + ilości w g). WczytajOstatniImport ładuje data/import/ostatni.json. Tint chart bez ilości = komunikat, bez zmiany składu.</t>
+          <t>Makro ImportujZPdf: natychmiast okno Windows (jak Eksplorator), filtr PDF. WczytajOstatniImport ładuje data/import/ostatni.json. Anulowanie i tint chart bez ilości = komunikat, bez zmiany składu.</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Wskaż PDF przyciskiem albo: Narzędzia → Makra → ImportujZPdf</t>
+          <t>Przycisk otwiera okno Windows (jak Eksplorator). Anulowanie nie czyści składu.</t>
         </is>
       </c>
     </row>
@@ -1980,7 +1980,7 @@
     <row r="39">
       <c r="A39" s="25" t="inlineStr">
         <is>
-          <t>Przykład testowy: data/import/przyklad_receptura_test.pdf. Przewodniki tint chart (bez kolumny ilości) nie są recepturą — pojawi się „nie znaleziono receptury”, skład nie zostanie wyczyszczony.</t>
+          <t>Przycisk Importuj otwiera natywne okno Windows (PDF). Anulowanie nie czyści składu. Przykład testowy: data/import/przyklad_receptura_test.pdf. Przewodniki tint chart (bez kolumny ilości) nie są recepturą — pojawi się „nie znaleziono receptury”.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Show the Calc FilePicker immediately when importing a recipe PDF.
</commit_message>
<xml_diff>
--- a/receptury-lakiery/RECEPTURY_LAKIERY.xlsx
+++ b/receptury-lakiery/RECEPTURY_LAKIERY.xlsx
@@ -1949,7 +1949,7 @@
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Przycisk otwiera okno Windows (jak Eksplorator). Anulowanie nie czyści składu.</t>
+          <t>Przycisk Importuj → od razu okno Otwórz (PDF). Gdy martwy: Narzędzia→Makra→ImportujZPdf.</t>
         </is>
       </c>
     </row>
@@ -1980,7 +1980,7 @@
     <row r="39">
       <c r="A39" s="25" t="inlineStr">
         <is>
-          <t>Przycisk Importuj otwiera natywne okno Windows (PDF). Anulowanie nie czyści składu. Przykład testowy: data/import/przyklad_receptura_test.pdf. Przewodniki tint chart (bez kolumny ilości) nie są recepturą — pojawi się „nie znaleziono receptury”.</t>
+          <t>Kliknij Importuj recepturę z PDF — od razu otworzy się okno Otwórz (jak Eksplorator), filtr PDF. Gdy przycisk nie działa: Narzędzia → Makra → Uruchom makro → Standard → modReceptury → ImportujZPdf. Przykład: data/import/przyklad_receptura_test.pdf. Tint chart bez ilości = „nie znaleziono receptury”.</t>
         </is>
       </c>
     </row>

</xml_diff>